<commit_message>
Publish Issue #5: callback-first + night-call-log callback columns
</commit_message>
<xml_diff>
--- a/offers/night-call-log/night-call-log.xlsx
+++ b/offers/night-call-log/night-call-log.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,7 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font/>
   </fonts>
   <fills count="3">
     <fill>
@@ -59,12 +60,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -457,8 +459,13 @@
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="21" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="44" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,6 +599,31 @@
           <t>logged_by</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>callback_attempts</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>callback_owner</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>last_callback_at</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>callback_outcome</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>ok_to_text</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -718,7 +750,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="12">
     <dataValidation sqref="X2:X1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Unbooked calls only. One code from the Issue #4 list; leave blank on booked calls." type="list">
       <formula1>"A_not_customer,B_existing_job,C_outside_area,D_work_we_dont_do,E_fee_declined,F_wanted_price_first,G_no_slot_that_worked,H_calling_back,I_needs_decider,J_other_quotes,Other"</formula1>
     </dataValidation>
@@ -746,6 +778,15 @@
     <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Use one value from the dropdown." type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
+    <dataValidation sqref="AA2:AA1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="0 to 3. Three tries max is our suggestion." type="list">
+      <formula1>"0,1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD2:AD1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Use one of the four callback outcomes." type="list">
+      <formula1>"Booked,Not booked (new code if the reason changed),No answer after all tries,Asked not to be contacted"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE2:AE1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Y or N. Ask on the first callback." type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -757,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1029,6 +1070,232 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Callbacks (calls coded H, E, F, J; same week as the call date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Calls with at least one callback attempt</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Total callback attempts</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*IFERROR(VALUE(Log!$AA$2:$AA$1000&amp;""),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Callback outcomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Booked</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Not booked (new code if the reason changed)</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="Not booked (new code if the reason changed)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>No answer after all tries</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="No answer after all tries"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Asked not to be contacted</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="Asked not to be contacted"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Callbacks booked</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>By code: attempted / booked</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>H_calling_back — callbacks attempted</t>
+        </is>
+      </c>
+      <c r="B40">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="H_calling_back")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>H_calling_back — callbacks booked</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="H_calling_back")*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>E_fee_declined — callbacks attempted</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="E_fee_declined")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>E_fee_declined — callbacks booked</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="E_fee_declined")*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>F_wanted_price_first — callbacks attempted</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="F_wanted_price_first")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>F_wanted_price_first — callbacks booked</t>
+        </is>
+      </c>
+      <c r="B45">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="F_wanted_price_first")*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>J_other_quotes — callbacks attempted</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="J_other_quotes")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>J_other_quotes — callbacks booked</t>
+        </is>
+      </c>
+      <c r="B47">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$X$2:$X$1000="J_other_quotes")*(Log!$AD$2:$AD$1000="Booked"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>H/E/F/J calls with no callback attempt yet (nobody tried)</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(((Log!$X$2:$X$1000="H_calling_back")+(Log!$X$2:$X$1000="E_fee_declined")+(Log!$X$2:$X$1000="F_wanted_price_first")+(Log!$X$2:$X$1000="J_other_quotes"))&gt;0)*(1-((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Callback logged on a code not on the callback list (A–D, G, I, Other, or blank)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(((Log!$X$2:$X$1000="H_calling_back")+(Log!$X$2:$X$1000="E_fee_declined")+(Log!$X$2:$X$1000="F_wanted_price_first")+(Log!$X$2:$X$1000="J_other_quotes"))=0)*(((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"")*((Log!$AA$2:$AA$1000&amp;"")&lt;&gt;"0")+(Log!$AD$2:$AD$1000&lt;&gt;"")&gt;0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>"Asked not to be contacted" rows with ok_to_text = Y (should be 0 — stop means stop)</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>SUMPRODUCT((Log!$A$2:$A$1000&lt;&gt;"EXAMPLE")*(Log!$B$2:$B$1000&lt;&gt;"")*(Log!$B$2:$B$1000&gt;=$B$2)*(Log!$B$2:$B$1000&lt;=$B$3)*(Log!$AD$2:$AD$1000="Asked not to be contacted")*(Log!$AE$2:$AE$1000="Y"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>